<commit_message>
(NCIOCPL#124) Fixed data errors for citations and language toggle.
</commit_message>
<xml_diff>
--- a/test-data/citations-data.xlsx
+++ b/test-data/citations-data.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="21328"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AB4F7AF-6C93-49A4-A32E-957E2D827E5E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85462BB2-4359-42CE-9A5A-876799E7874D}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15" yWindow="0" windowWidth="19185" windowHeight="10200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pages_with_citations" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="48">
   <si>
     <t>path</t>
   </si>
@@ -53,9 +53,6 @@
     <t>/espanol/noticias/comunicados-de-prensa/2018/leucemia-llc-ibrutinib-estudio</t>
   </si>
   <si>
-    <t>Referencias</t>
-  </si>
-  <si>
     <t>Selected References</t>
   </si>
   <si>
@@ -162,6 +159,12 @@
   </si>
   <si>
     <t>Video</t>
+  </si>
+  <si>
+    <t>Bibliografía selecta</t>
+  </si>
+  <si>
+    <t>Bibliografía</t>
   </si>
 </sst>
 </file>
@@ -522,7 +525,7 @@
         <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -536,10 +539,10 @@
         <v>4</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -553,15 +556,15 @@
         <v>4</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s">
         <v>3</v>
@@ -570,10 +573,10 @@
         <v>5</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -581,50 +584,50 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
       </c>
       <c r="D5" t="s">
-        <v>10</v>
+        <v>47</v>
       </c>
       <c r="E5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" t="s">
         <v>13</v>
       </c>
-      <c r="C6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D6" t="s">
-        <v>14</v>
-      </c>
       <c r="E6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
         <v>4</v>
       </c>
       <c r="D7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -659,10 +662,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" t="s">
         <v>18</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
@@ -670,10 +673,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
@@ -681,10 +684,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
         <v>22</v>
-      </c>
-      <c r="B4" t="s">
-        <v>23</v>
       </c>
       <c r="C4" t="s">
         <v>4</v>
@@ -692,10 +695,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" t="s">
         <v>24</v>
-      </c>
-      <c r="B5" t="s">
-        <v>25</v>
       </c>
       <c r="C5" t="s">
         <v>4</v>
@@ -703,10 +706,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" t="s">
         <v>26</v>
-      </c>
-      <c r="B6" t="s">
-        <v>27</v>
       </c>
       <c r="C6" t="s">
         <v>4</v>
@@ -714,10 +717,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
@@ -725,10 +728,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s">
         <v>29</v>
-      </c>
-      <c r="B8" t="s">
-        <v>30</v>
       </c>
       <c r="C8" t="s">
         <v>4</v>
@@ -736,10 +739,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
         <v>5</v>
@@ -747,10 +750,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
         <v>4</v>
@@ -758,10 +761,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
         <v>33</v>
-      </c>
-      <c r="B11" t="s">
-        <v>34</v>
       </c>
       <c r="C11" t="s">
         <v>4</v>
@@ -769,10 +772,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C12" t="s">
         <v>4</v>
@@ -780,10 +783,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C13" t="s">
         <v>5</v>
@@ -791,10 +794,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" t="s">
         <v>38</v>
-      </c>
-      <c r="B14" t="s">
-        <v>39</v>
       </c>
       <c r="C14" t="s">
         <v>4</v>
@@ -802,10 +805,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C15" t="s">
         <v>5</v>
@@ -813,10 +816,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" t="s">
         <v>42</v>
-      </c>
-      <c r="B16" t="s">
-        <v>43</v>
       </c>
       <c r="C16" t="s">
         <v>4</v>
@@ -824,10 +827,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C17" t="s">
         <v>5</v>
@@ -835,10 +838,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" t="s">
         <v>45</v>
-      </c>
-      <c r="B18" t="s">
-        <v>46</v>
       </c>
       <c r="C18" t="s">
         <v>4</v>

</xml_diff>